<commit_message>
feat(snr): SNR = BA "Net revenue" definition; Skybase GAR primitive; #166 psm3 regression fix (#170)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-02/skybase_settlement_february_2026.xlsx
+++ b/settlements/skybase/2026-02/skybase_settlement_february_2026.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -511,130 +511,140 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>207894.1499334339</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>+ governance_accessibility_rewards (0.01 × SNR 2026-01 = 9218713.81273186308887946403 (sky_total generated sky_total))</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>92187.13812731863</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" s="4" t="n">
+        <v>300081.2880607526</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-02-01 → 2026-02-28 (28 days)</t>
-        </is>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ethereum=24558867</t>
+          <t>2026-02-01 → 2026-02-28 (28 days)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-15T11:05:12+00:00</t>
+          <t>ethereum=24558867</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-05T23:50:46+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>